<commit_message>
footer - mermaid fixes
</commit_message>
<xml_diff>
--- a/temp/pages/StructureDefinition-WRCondition.xlsx
+++ b/temp/pages/StructureDefinition-WRCondition.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-09-13T22:44:23+00:00</t>
+    <t>2025-09-27T21:51:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -72,7 +72,7 @@
     <t>Contact</t>
   </si>
   <si>
-    <t>Andrew Rose LPC (http://wrig.corisystem.org)</t>
+    <t>Andrew Rose LPC (https://wrig.corisystem.org)</t>
   </si>
   <si>
     <t>Jurisdiction</t>

</xml_diff>